<commit_message>
Implement leakage-free QSAR workflow with train-only preprocessing
</commit_message>
<xml_diff>
--- a/output/publication_tables/Publication_Tables.xlsx
+++ b/output/publication_tables/Publication_Tables.xlsx
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6396785889070081</v>
+        <v>0.6462493440520147</v>
       </c>
       <c r="C6" t="n">
         <v/>
@@ -730,13 +730,13 @@
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>0.6447982987100336</v>
+        <v>0.647168960213711</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7923155543012507</v>
+        <v>0.7896671203237712</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5709156907869247</v>
+        <v>0.5633688279301922</v>
       </c>
     </row>
   </sheetData>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.35063145</v>
+        <v>0.35175014</v>
       </c>
     </row>
     <row r="3">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1810794</v>
+        <v>0.1948334</v>
       </c>
     </row>
     <row r="4">
@@ -792,67 +792,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.06731158</v>
+        <v>0.07120600000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FractionCSP3</t>
+          <t>Chi2v</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.04906383</v>
+        <v>0.052803725</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SMR_VSA10</t>
+          <t>SlogP_VSA12</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.049040552</v>
+        <v>0.049540598</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kappa2</t>
+          <t>FractionCSP3</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.04831299</v>
+        <v>0.04901301</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SlogP_VSA12</t>
+          <t>SMR_VSA10</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.04758621</v>
+        <v>0.047656544</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BertzCT</t>
+          <t>Kappa2</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.042633574</v>
+        <v>0.045960013</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SlogP_VSA2</t>
+          <t>BertzCT</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.041129157</v>
+        <v>0.043254584</v>
       </c>
     </row>
     <row r="11">
@@ -862,37 +862,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.040415347</v>
+        <v>0.04320746</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Chi2v</t>
+          <t>SlogP_VSA2</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.040397625</v>
+        <v>0.04038709</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chi3v</t>
+          <t>PEOE_VSA6</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.040154237</v>
+        <v>0.033345286</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PEOE_VSA6</t>
+          <t>NHOHCount</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.028096495</v>
+        <v>0.029014153</v>
       </c>
     </row>
     <row r="15">
@@ -902,37 +902,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.024929766</v>
+        <v>0.026990302</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SPS</t>
+          <t>MinEStateIndex</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.020465571</v>
+        <v>0.022115791</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SMR_VSA9</t>
+          <t>AvgIpc</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.019101614</v>
+        <v>0.021856807</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Kappa3</t>
+          <t>SPS</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.01909426</v>
+        <v>0.021422917</v>
       </c>
     </row>
     <row r="19">
@@ -942,27 +942,27 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.01851204</v>
+        <v>0.020217596</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SMR_VSA1</t>
+          <t>Kappa3</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.017237213</v>
+        <v>0.019940523</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PEOE_VSA1</t>
+          <t>fr_Ar_OH</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.017214933</v>
+        <v>0.01949143</v>
       </c>
     </row>
   </sheetData>
@@ -1150,25 +1150,25 @@
         <v>20</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.2137455812019464</v>
+        <v>-0.2118765802735946</v>
       </c>
       <c r="C3" t="n">
-        <v>0.02293962059778312</v>
+        <v>0.02244548683091611</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.2537796925748418</v>
+        <v>-0.2578855170719262</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.2275653802423178</v>
+        <v>-0.2243802439388308</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.2208512221285936</v>
+        <v>-0.2205729264642481</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1961043754913059</v>
+        <v>-0.1937374262575705</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1765780090747704</v>
+        <v>-0.1723723894583934</v>
       </c>
     </row>
   </sheetData>

</xml_diff>